<commit_message>
Convert score columns to pure numbers and compute policy/instrument scores
Co-authored-by: Vaibhav <shivrain@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/4p-index/STP_Decreto-37-1999_EIA-Decree_4P-Index.xlsx
+++ b/4p-index/STP_Decreto-37-1999_EIA-Decree_4P-Index.xlsx
@@ -636,12 +636,12 @@
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>[auto]</t>
+          <t>0.9</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>1 (Regulatory)</t>
+          <t>1</t>
         </is>
       </c>
       <c r="Q2" s="2" t="inlineStr">
@@ -671,12 +671,12 @@
       </c>
       <c r="V2" s="2" t="inlineStr">
         <is>
-          <t>[auto]</t>
+          <t>0.875</t>
         </is>
       </c>
       <c r="W2" s="2" t="inlineStr">
         <is>
-          <t>No explicit mention of 'plastics'; qualifies via Annex I items 8 (chemical/industrial manufacturing, potentially including plastics production/processing), 11 (hazardous waste) and 12 (municipal/industrial waste landfill, treatment and disposal — directly covers plastic waste streams) — plastics-relevance criteria (b)/(c). Screening (Art. 5) and the full EIA study (Art. 6) are combined into a single row per Rule 10, as they form one integrated mandatory assessment procedure.</t>
+          <t>Instrument type: Regulatory (1). No explicit mention of 'plastics'; qualifies via Annex I items 8 (chemical/industrial manufacturing, potentially including plastics production/processing), 11 (hazardous waste) and 12 (municipal/industrial waste landfill, treatment and disposal — directly covers plastic waste streams) — plastics-relevance criteria (b)/(c). Screening (Art. 5) and the full EIA study (Art. 6) are combined into a single row per Rule 10, as they form one integrated mandatory assessment procedure.</t>
         </is>
       </c>
     </row>
@@ -749,12 +749,12 @@
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>[auto]</t>
+          <t>0.74</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>0.20 (Governance &amp; coordination)</t>
+          <t>0.2</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
@@ -784,12 +784,12 @@
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>[auto]</t>
+          <t>0.35</t>
         </is>
       </c>
       <c r="W3" s="2" t="inlineStr">
         <is>
-          <t>Applies to the same set of Annex-I-listed activities as Row 1, including plastics-relevant waste/industrial facilities; public hearings are discretionary depending on project scale (Art. 7.º(4)) — coded as a governance/participation instrument rather than Regulatory since it does not itself ban, standardise or economically incentivise anything.</t>
+          <t>Instrument type: Governance &amp; coordination (0.2). Applies to the same set of Annex-I-listed activities as Row 1, including plastics-relevant waste/industrial facilities; public hearings are discretionary depending on project scale (Art. 7.º(4)) — coded as a governance/participation instrument rather than Regulatory since it does not itself ban, standardise or economically incentivise anything.</t>
         </is>
       </c>
     </row>
@@ -862,12 +862,12 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>[auto]</t>
+          <t>0.9</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>1 (Regulatory)</t>
+          <t>1</t>
         </is>
       </c>
       <c r="Q4" s="2" t="inlineStr">
@@ -897,12 +897,12 @@
       </c>
       <c r="V4" s="2" t="inlineStr">
         <is>
-          <t>[auto]</t>
+          <t>1</t>
         </is>
       </c>
       <c r="W4" s="2" t="inlineStr">
         <is>
-          <t>Functions as the core 'upstream gatekeeping' mechanism referenced in the policy summary — makes the environmental licence a legal precondition for all other sectoral licences, e.g. industrial operating licences for plastics-processing or packaging facilities.</t>
+          <t>Instrument type: Regulatory (1). Functions as the core 'upstream gatekeeping' mechanism referenced in the policy summary — makes the environmental licence a legal precondition for all other sectoral licences, e.g. industrial operating licences for plastics-processing or packaging facilities.</t>
         </is>
       </c>
     </row>
@@ -975,12 +975,12 @@
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>[auto]</t>
+          <t>0.9</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>1 (Regulatory)</t>
+          <t>1</t>
         </is>
       </c>
       <c r="Q5" s="2" t="inlineStr">
@@ -1010,12 +1010,12 @@
       </c>
       <c r="V5" s="2" t="inlineStr">
         <is>
-          <t>[auto]</t>
+          <t>0.625</t>
         </is>
       </c>
       <c r="W5" s="2" t="inlineStr">
         <is>
-          <t>A sunset clause preventing indefinite 'banking' of unused environmental licences; relevant to plastics-processing or waste facilities that might otherwise hold a licence without updated impact data.</t>
+          <t>Instrument type: Regulatory (1). A sunset clause preventing indefinite 'banking' of unused environmental licences; relevant to plastics-processing or waste facilities that might otherwise hold a licence without updated impact data.</t>
         </is>
       </c>
     </row>
@@ -1088,12 +1088,12 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>[auto]</t>
+          <t>0.9</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>1 (Regulatory)</t>
+          <t>1</t>
         </is>
       </c>
       <c r="Q6" s="2" t="inlineStr">
@@ -1123,12 +1123,12 @@
       </c>
       <c r="V6" s="2" t="inlineStr">
         <is>
-          <t>[auto]</t>
+          <t>1</t>
         </is>
       </c>
       <c r="W6" s="2" t="inlineStr">
         <is>
-          <t>Mixed governance (professional registry) and economic (registration fee, Annex III) instrument; scored as Regulatory (1.0) per Rule 10 because the core requirement — that only registered consultants may conduct EIA studies — is a mandatory professional/technical standard, with the fee treated as an ancillary economic component. Relevant to plastics only insofar as it underpins the quality/credibility of EIA studies for plastics-relevant facilities (criterion c).</t>
+          <t>Instrument type: Regulatory (1). Mixed governance (professional registry) and economic (registration fee, Annex III) instrument; scored as Regulatory (1.0) per Rule 10 because the core requirement — that only registered consultants may conduct EIA studies — is a mandatory professional/technical standard, with the fee treated as an ancillary economic component. Relevant to plastics only insofar as it underpins the quality/credibility of EIA studies for plastics-relevant facilities (criterion c).</t>
         </is>
       </c>
     </row>
@@ -1201,12 +1201,12 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>[auto]</t>
+          <t>0.74</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>0.20 (Governance &amp; coordination)</t>
+          <t>0.2</t>
         </is>
       </c>
       <c r="Q7" s="2" t="inlineStr">
@@ -1236,12 +1236,12 @@
       </c>
       <c r="V7" s="2" t="inlineStr">
         <is>
-          <t>[auto]</t>
+          <t>0.35</t>
         </is>
       </c>
       <c r="W7" s="2" t="inlineStr">
         <is>
-          <t>Coded as a standalone governance/monitoring instrument (0.20) rather than folded into the Regulatory rows, consistent with Rule 11 (assignment of enforcement/monitoring responsibilities). Applies to any licensed or unlicensed activity capable of causing environmental damage, including plastics-relevant waste or industrial facilities.</t>
+          <t>Instrument type: Governance &amp; coordination (0.2). Coded as a standalone governance/monitoring instrument (0.20) rather than folded into the Regulatory rows, consistent with Rule 11 (assignment of enforcement/monitoring responsibilities). Applies to any licensed or unlicensed activity capable of causing environmental damage, including plastics-relevant waste or industrial facilities.</t>
         </is>
       </c>
     </row>
@@ -1314,12 +1314,12 @@
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>[auto]</t>
+          <t>0.9</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>1 (Regulatory)</t>
+          <t>1</t>
         </is>
       </c>
       <c r="Q8" s="2" t="inlineStr">
@@ -1349,12 +1349,12 @@
       </c>
       <c r="V8" s="2" t="inlineStr">
         <is>
-          <t>[auto]</t>
+          <t>0.75</t>
         </is>
       </c>
       <c r="W8" s="2" t="inlineStr">
         <is>
-          <t>Directly enforces the EIA/licensing gatekeeping regime (Rows 1 and 3) against non-compliant proponents, including those operating plastics-processing, packaging or waste-treatment facilities without required EIA clearance. Mixed instrument: mandatory liability (in force) combined with a discretionary embargo enabling power — coded S = 1 overall because the liability rule itself uses mandatory language; flagged here as a borderline case.</t>
+          <t>Instrument type: Regulatory (1). Directly enforces the EIA/licensing gatekeeping regime (Rows 1 and 3) against non-compliant proponents, including those operating plastics-processing, packaging or waste-treatment facilities without required EIA clearance. Mixed instrument: mandatory liability (in force) combined with a discretionary embargo enabling power — coded S = 1 overall because the liability rule itself uses mandatory language; flagged here as a borderline case.</t>
         </is>
       </c>
     </row>
@@ -1427,12 +1427,12 @@
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>[auto]</t>
+          <t>0.82</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>0.60 (Economic)</t>
+          <t>0.6</t>
         </is>
       </c>
       <c r="Q9" s="2" t="inlineStr">
@@ -1462,12 +1462,12 @@
       </c>
       <c r="V9" s="2" t="inlineStr">
         <is>
-          <t>[auto]</t>
+          <t>0.55</t>
         </is>
       </c>
       <c r="W9" s="2" t="inlineStr">
         <is>
-          <t>Ring-fenced/self-generated funding: fees are explicitly earmarked to finance the EIA process itself (Annex II(3); same wording in Annex III(3) for consultant registration fees) — this underpins policy-level Col M = 1. Applies to any project subject to EIA (including plastics-relevant facilities under Annex I), calculated as a percentage of project value rather than as a plastics-specific levy.</t>
+          <t>Instrument type: Economic (0.6). Ring-fenced/self-generated funding: fees are explicitly earmarked to finance the EIA process itself (Annex II(3); same wording in Annex III(3) for consultant registration fees) — this underpins policy-level Col M = 1. Applies to any project subject to EIA (including plastics-relevant facilities under Annex I), calculated as a percentage of project value rather than as a plastics-specific levy.</t>
         </is>
       </c>
     </row>

</xml_diff>